<commit_message>
TP1 Orga de datos
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fernando\Desktop\Facultad\2026\Primer-Cuatrimestre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D832AA-65DC-4393-BD40-08DCC175DB71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC56904-ACDC-4ACA-8A86-EBE39DED5A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E120C665-BE77-45F5-8364-6C3ECB26DAEB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>LUNES</t>
   </si>
@@ -75,10 +75,6 @@
   </si>
   <si>
     <t>MIÉRCOLES</t>
-  </si>
-  <si>
-    <t>17:00-18:00
-Aula 106</t>
   </si>
   <si>
     <t>8:00-10:00
@@ -102,10 +98,16 @@
     <t>14:00-18:00 TP - Aula 01</t>
   </si>
   <si>
-    <t>14:00-17:00 TP - Aula 205</t>
-  </si>
-  <si>
-    <t>14:00-17:00 TP - Aula 02</t>
+    <t>13:00-16:00 TP - Aula 02</t>
+  </si>
+  <si>
+    <t>13:00-16:00 TP - Aula 205</t>
+  </si>
+  <si>
+    <t>Economía del conocimiento</t>
+  </si>
+  <si>
+    <t>18:00-21:00 TP-Aula 103</t>
   </si>
 </sst>
 </file>
@@ -129,7 +131,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,6 +174,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF77171"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -308,9 +316,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -319,6 +326,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -337,79 +383,67 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -427,27 +461,38 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,6 +502,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFF77171"/>
       <color rgb="FFFFFDAD"/>
     </mruColors>
   </colors>
@@ -788,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACA7E160-EBC7-43BF-A8A5-B19AEC632419}">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" customWidth="1"/>
@@ -799,344 +845,378 @@
   <sheetData>
     <row r="1" spans="1:10" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="48" t="s">
+      <c r="E2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="48" t="s">
+      <c r="F2" s="7" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="51">
+      <c r="A3" s="9">
         <v>0.33333333333333331</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="49" t="s">
+      <c r="B3" s="1"/>
+      <c r="E3" s="52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="H3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="17"/>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="2"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="62">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="9">
+        <v>0.375</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="D5" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="53"/>
+      <c r="F5" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="58" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="59"/>
+      <c r="J5" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>0.39583333333333298</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="33"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="8"/>
+    </row>
+    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="H7" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="41"/>
+      <c r="J7" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>0.4375</v>
+      </c>
+      <c r="B8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="2"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="9">
+        <v>0.45833333333333298</v>
+      </c>
+      <c r="B9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="2"/>
+      <c r="H9" s="44" t="s">
+        <v>4</v>
+      </c>
+      <c r="I9" s="45"/>
+      <c r="J9" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9">
+        <v>0.47916666666666702</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="2"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="8"/>
+    </row>
+    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="E11" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="H11" s="48" t="s">
+        <v>8</v>
+      </c>
+      <c r="I11" s="49"/>
+      <c r="J11" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9">
+        <v>0.52083333333333304</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="E12" s="56"/>
+      <c r="F12" s="2"/>
+      <c r="H12" s="50"/>
+      <c r="I12" s="51"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
+        <v>0.54166666666666696</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="D13" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="56"/>
+      <c r="F13" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" s="35"/>
+      <c r="J13" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9">
+        <v>0.5625</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="29"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
+        <v>0.58333333333333304</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="30"/>
+      <c r="E15" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="51">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="51">
-        <v>0.375</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="32"/>
-      <c r="J5" s="50">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="51">
-        <v>0.39583333333333298</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="28"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="50"/>
-    </row>
-    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="51">
-        <v>0.41666666666666702</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
-      <c r="E7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="H7" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7" s="34"/>
-      <c r="J7" s="50">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="51">
-        <v>0.4375</v>
-      </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="3"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="50"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="51">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="3"/>
-      <c r="H9" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="I9" s="38"/>
-      <c r="J9" s="50">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="51">
-        <v>0.47916666666666702</v>
-      </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="3"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="50"/>
-    </row>
-    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="51">
-        <v>0.5</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="3"/>
-      <c r="H11" s="40" t="s">
-        <v>8</v>
-      </c>
-      <c r="I11" s="41"/>
-      <c r="J11" s="50">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="51">
-        <v>0.52083333333333304</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="3"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="50"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="51">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="47"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="3"/>
-      <c r="H13" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="I13" s="20"/>
-      <c r="J13" s="50">
+      <c r="F15" s="29"/>
+      <c r="H15" s="38" t="s">
+        <v>5</v>
+      </c>
+      <c r="I15" s="32"/>
+      <c r="J15" s="8">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="51">
-        <v>0.5625</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="3"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="50"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="51">
-        <v>0.58333333333333304</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="I15" s="26"/>
-      <c r="J15" s="50">
-        <v>3</v>
-      </c>
-    </row>
     <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="51">
+      <c r="A16" s="9">
         <v>0.60416666666666696</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="12"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="24"/>
       <c r="D16" s="30"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="30"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="50"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="29"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="51">
+      <c r="A17" s="9">
         <v>0.625</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="12"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="30"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="30"/>
-      <c r="J17" s="50"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="29"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="51">
+      <c r="A18" s="9">
         <v>0.64583333333333404</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="30"/>
-      <c r="J18" s="50">
-        <f>+SUM(J5:J13)</f>
-        <v>21</v>
+      <c r="B18" s="1"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="61"/>
+      <c r="J18" s="8">
+        <f>+SUM(J4:J13)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="51">
+      <c r="A19" s="9">
         <v>0.66666666666666696</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="30"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="10"/>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="51">
+      <c r="A20" s="9">
         <v>0.6875</v>
       </c>
       <c r="B20" s="27"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="46"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="51">
+      <c r="C20" s="24"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
+    </row>
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9">
         <v>0.70833333333333404</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="45"/>
-      <c r="F21" s="3"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="2"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="51">
+      <c r="A22" s="9">
         <v>0.72916666666666696</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="3"/>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="51">
+      <c r="B22" s="1"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="2"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="9">
         <v>0.75</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="7"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
+      <c r="A24" s="9">
+        <v>0.77083333333333304</v>
+      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="14"/>
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="9">
+        <v>0.79166666666666596</v>
+      </c>
+      <c r="B25" s="1"/>
+      <c r="C25" s="14"/>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="9">
+        <v>0.812499999999999</v>
+      </c>
+      <c r="B26" s="1"/>
+      <c r="C26" s="14"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="9">
+        <v>0.83333333333333204</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="14"/>
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="9">
+        <v>0.85416666666666496</v>
+      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="15"/>
+      <c r="F28" s="2"/>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="9">
+        <v>0.874999999999998</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="E15:E18"/>
+    <mergeCell ref="H5:I6"/>
+    <mergeCell ref="F13:F18"/>
+    <mergeCell ref="C23:C28"/>
+    <mergeCell ref="H3:I4"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C15:C22"/>
+    <mergeCell ref="E7:E10"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="D13:D18"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="H13:I14"/>
     <mergeCell ref="H15:I16"/>
-    <mergeCell ref="F15:F20"/>
     <mergeCell ref="H7:I8"/>
     <mergeCell ref="H9:I10"/>
     <mergeCell ref="H11:I12"/>
     <mergeCell ref="E3:E6"/>
     <mergeCell ref="E11:E14"/>
-    <mergeCell ref="E15:E18"/>
-    <mergeCell ref="H5:I6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C15:C22"/>
-    <mergeCell ref="D15:D20"/>
-    <mergeCell ref="E7:E10"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="D21:D22"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>